<commit_message>
APK 3.16.0: columna RESPONSABLE en carga masiva de equipos (plantilla e importacion)
</commit_message>
<xml_diff>
--- a/excel_ejemplo/equipos.xlsx
+++ b/excel_ejemplo/equipos.xlsx
@@ -18,55 +18,60 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>RESPONSABLE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>DNI</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>HOSTNAME</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DIR. IP</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>UBICACIÓN FISICA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>EQUIPO</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>COD. INVENTARIO</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>SERIE DE EQUIPO</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>MARCA</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>MODELO</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>CONTRATO DE ARRENDAMIENTO</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
@@ -80,55 +85,60 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Juan Carlos Perez Gomez</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>45211365</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>LAP-JP-01</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>192.168.10.11</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Oficina 101 - Piso 1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>INV-2026-0001</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>SRLP-JP-0001</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Lenovo</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>ThinkPad T14 Gen 3</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>CT-2026-0147</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
@@ -142,55 +152,60 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Juan Carlos Perez Gomez</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>45211365</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>LAP-JP-02</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>192.168.10.12</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Oficina 101 - Piso 1</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>INV-2026-0002</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>SRLP-JP-0002</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Dell</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Latitude 5440</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>CT-2026-0147</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>En uso</t>
         </is>
@@ -204,55 +219,60 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Maria Fernanda Lopez</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>45211366</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>LAP-ML-01</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>192.168.10.21</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Oficina 202 - Piso 2</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Laptop</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>INV-2026-0003</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>SRLP-ML-0001</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>HP</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>EliteBook 840</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>CT-2026-0201</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
@@ -266,55 +286,60 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Carlos Alberto Ramirez</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>45211367</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>DESK-CR-01</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>192.168.10.31</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Almacen Sur</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Desktop</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>INV-2026-0004</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>SRDS-CR-0001</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>HP</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>ProDesk 400</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>CT-2026-0301</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>En uso</t>
         </is>
@@ -328,55 +353,60 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Ana Lucia Torres</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>45211368</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>IMPR-AT-01</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>192.168.10.41</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Planta - Produccion</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Impresora</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>INV-2026-0005</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>SRIM-AT-0001</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Epson</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>EcoTank L5290</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>CT-2026-0401</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>

</xml_diff>